<commit_message>
2026-08-21 리포트 보정: 4종목(SPCX/LUNR/VOYG/MDA) 등락률 데이터 보완
클라우드 실행에서 확인 필요로 남았던 4종목의 이번주 등락률을 Yahoo Finance
차트 API로 직접 확인해 채움. Intuitive Machines(LUNR)이 유일한 상승 종목
(+2.85%)으로 확인되어 상승/하락 상위 요약도 함께 수정. 발표 대본도 동일하게
갱신.
</commit_message>
<xml_diff>
--- a/reports/2026-08-21-tiger-space-etf-weekly.xlsx
+++ b/reports/2026-08-21-tiger-space-etf-weekly.xlsx
@@ -537,21 +537,21 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>이번 주 상승 상위: 해당 종목 없음 (등락률이 확인된 6종목 모두 하락)</t>
+          <t>이번 주 상승 상위: Intuitive Machines(LUNR) +2.85% (유일한 상승 종목)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>이번 주 하락 상위 3개: Firefly Aerospace(FLY) -20.07%, AST SpaceMobile(ASTS) -9.74%, Planet Labs(PL) -8.61%</t>
+          <t>이번 주 하락 상위 3개: Firefly Aerospace(FLY) -20.07%, Voyager Technologies(VOYG) -12.19%, MDA Space(MDA) -10.23%</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>조사 대상 10종목 중 SpaceX·Intuitive Machines·Voyager Technologies·MDA Space 4종목은 등락률 데이터 확인 필요로 순위 산정에서 제외함. 확인된 6종목은 전원 하락(상승 종목 없음).</t>
+          <t>조사 대상 10종목 중 상승 종목은 Intuitive Machines(LUNR) 1개뿐이며, 나머지 9종목은 모두 하락.</t>
         </is>
       </c>
     </row>
@@ -617,10 +617,8 @@
       <c r="B13" s="9" t="n">
         <v>0.2477</v>
       </c>
-      <c r="C13" s="10" t="inlineStr">
-        <is>
-          <t>확인 필요</t>
-        </is>
+      <c r="C13" s="9" t="n">
+        <v>-0.0516</v>
       </c>
       <c r="D13" s="11" t="n">
         <v>134</v>
@@ -691,10 +689,8 @@
       <c r="B16" s="9" t="n">
         <v>0.1296</v>
       </c>
-      <c r="C16" s="10" t="inlineStr">
-        <is>
-          <t>확인 필요</t>
-        </is>
+      <c r="C16" s="9" t="n">
+        <v>0.0285</v>
       </c>
       <c r="D16" s="11" t="n">
         <v>18.06</v>
@@ -789,10 +785,8 @@
       <c r="B20" s="9" t="n">
         <v>0.0336</v>
       </c>
-      <c r="C20" s="10" t="inlineStr">
-        <is>
-          <t>확인 필요</t>
-        </is>
+      <c r="C20" s="9" t="n">
+        <v>-0.1219</v>
       </c>
       <c r="D20" s="11" t="n">
         <v>38.88</v>
@@ -815,15 +809,11 @@
       <c r="B21" s="9" t="n">
         <v>0.0332</v>
       </c>
-      <c r="C21" s="10" t="inlineStr">
-        <is>
-          <t>확인 필요</t>
-        </is>
-      </c>
-      <c r="D21" s="10" t="inlineStr">
-        <is>
-          <t>확인 필요</t>
-        </is>
+      <c r="C21" s="9" t="n">
+        <v>-0.1023</v>
+      </c>
+      <c r="D21" s="11" t="n">
+        <v>31.25</v>
       </c>
       <c r="E21" s="12" t="n">
         <v>52.9</v>
@@ -861,7 +851,7 @@
     <row r="24">
       <c r="A24" s="13" t="inlineStr">
         <is>
-          <t>자료: 미래에셋자산운용 TIGER ETF 월간운용보고서(FactSheet, 2026년 7월 31일 기준) 및 investments.miraeasset.com/tigeretf 상세페이지(ETF 시장가격·순자산총액, 2026-08-21 조회), 언론보도·기업 IR 자료(개별종목 주가·이슈, WebSearch 기준 2026-08-20~21 조회). '확인 필요'로 표기된 항목은 신뢰할 수 있는 소스에서 값을 확정하지 못해 임의로 추정하지 않음. MDA Space 시가총액은 캐나다달러(TSX 기준) 표시금액을 근사 환율로 환산한 값이며, 비중 합계는 반올림으로 100%와 소폭 차이가 있을 수 있음.</t>
+          <t>자료: 미래에셋자산운용 TIGER ETF 월간운용보고서(FactSheet, 2026년 7월 31일 기준) 및 investments.miraeasset.com/tigeretf 상세페이지(ETF 시장가격·순자산총액, 2026-08-21 조회), 언론보도·기업 IR 자료(개별종목 주가·이슈, WebSearch 기준 2026-08-20~21 조회). '확인 필요'로 표기된 항목은 신뢰할 수 있는 소스에서 값을 확정하지 못해 임의로 추정하지 않음. MDA Space 시가총액은 캐나다달러(TSX 기준) 표시금액을 근사 환율로 환산한 값이며, 비중 합계는 반올림으로 100%와 소폭 차이가 있을 수 있음. SpaceX·Intuitive Machines·Voyager Technologies·MDA Space의 이번주 등락률(및 MDA 종가)은 Yahoo Finance 차트 데이터로 2026-08-21 추가 확인해 보완함.</t>
         </is>
       </c>
     </row>

</xml_diff>